<commit_message>
revised bib naming scheme
</commit_message>
<xml_diff>
--- a/ready-for-annotation/de/rotkaeppchen_khm-026_perrault.xlsx
+++ b/ready-for-annotation/de/rotkaeppchen_khm-026_perrault.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2451" uniqueCount="788">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2546" uniqueCount="788">
   <si>
     <t>ID</t>
   </si>
@@ -2917,9 +2917,8 @@
       <c r="F2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="9">
-        <f>IF(A2=1,"_",IF(C2="_","???",C2))</f>
-        <v/>
+      <c r="G2" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>12</v>
@@ -2948,9 +2947,8 @@
       <c r="F3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="9">
-        <f>IF(A3=1,"_",IF(C3="_","???",C3))</f>
-        <v/>
+      <c r="G3" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>12</v>
@@ -2979,9 +2977,8 @@
       <c r="F4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="9">
-        <f>IF(A4=1,"_",IF(C4="_","???",C4))</f>
-        <v/>
+      <c r="G4" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>12</v>
@@ -3010,9 +3007,8 @@
       <c r="F5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="9">
-        <f>IF(A5=1,"_",IF(C5="_","???",C5))</f>
-        <v/>
+      <c r="G5" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>12</v>
@@ -3041,9 +3037,8 @@
       <c r="F6" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="9">
-        <f>IF(A6=1,"_",IF(C6="_","???",C6))</f>
-        <v/>
+      <c r="G6" s="9" t="s">
+        <v>31</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>12</v>
@@ -3072,9 +3067,8 @@
       <c r="F7" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G7" s="9">
-        <f>IF(A7=1,"_",IF(C7="_","???",C7))</f>
-        <v/>
+      <c r="G7" s="9" t="s">
+        <v>35</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>12</v>
@@ -3103,9 +3097,8 @@
       <c r="F8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="9">
-        <f>IF(A8=1,"_",IF(C8="_","???",C8))</f>
-        <v/>
+      <c r="G8" s="9" t="s">
+        <v>39</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>12</v>
@@ -3134,9 +3127,8 @@
       <c r="F9" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="9">
-        <f>IF(A9=1,"_",IF(C9="_","???",C9))</f>
-        <v/>
+      <c r="G9" s="9" t="s">
+        <v>43</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>12</v>
@@ -3165,9 +3157,8 @@
       <c r="F10" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="G10" s="9">
-        <f>IF(A10=1,"_",IF(C10="_","???",C10))</f>
-        <v/>
+      <c r="G10" s="9" t="s">
+        <v>48</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>12</v>
@@ -3196,9 +3187,8 @@
       <c r="F11" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="G11" s="9">
-        <f>IF(A11=1,"_",IF(C11="_","???",C11))</f>
-        <v/>
+      <c r="G11" s="9" t="s">
+        <v>52</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>12</v>
@@ -3227,9 +3217,8 @@
       <c r="F12" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G12" s="9">
-        <f>IF(A12=1,"_",IF(C12="_","???",C12))</f>
-        <v/>
+      <c r="G12" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>12</v>
@@ -3258,9 +3247,8 @@
       <c r="F13" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="G13" s="9">
-        <f>IF(A13=1,"_",IF(C13="_","???",C13))</f>
-        <v/>
+      <c r="G13" s="9" t="s">
+        <v>59</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>12</v>
@@ -3289,9 +3277,8 @@
       <c r="F14" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="9">
-        <f>IF(A14=1,"_",IF(C14="_","???",C14))</f>
-        <v/>
+      <c r="G14" s="9" t="s">
+        <v>62</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>12</v>
@@ -3320,9 +3307,8 @@
       <c r="F15" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="G15" s="9">
-        <f>IF(A15=1,"_",IF(C15="_","???",C15))</f>
-        <v/>
+      <c r="G15" s="9" t="s">
+        <v>66</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>12</v>
@@ -3351,9 +3337,8 @@
       <c r="F16" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="G16" s="9">
-        <f>IF(A16=1,"_",IF(C16="_","???",C16))</f>
-        <v/>
+      <c r="G16" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>12</v>
@@ -3382,9 +3367,8 @@
       <c r="F17" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="G17" s="9">
-        <f>IF(A17=1,"_",IF(C17="_","???",C17))</f>
-        <v/>
+      <c r="G17" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H17" s="10" t="s">
         <v>12</v>
@@ -3413,9 +3397,8 @@
       <c r="F18" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="G18" s="9">
-        <f>IF(A18=1,"_",IF(C18="_","???",C18))</f>
-        <v/>
+      <c r="G18" s="9" t="s">
+        <v>77</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>12</v>
@@ -3444,9 +3427,8 @@
       <c r="F19" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="G19" s="9">
-        <f>IF(A19=1,"_",IF(C19="_","???",C19))</f>
-        <v/>
+      <c r="G19" s="9" t="s">
+        <v>81</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>12</v>
@@ -3475,9 +3457,8 @@
       <c r="F20" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="G20" s="9">
-        <f>IF(A20=1,"_",IF(C20="_","???",C20))</f>
-        <v/>
+      <c r="G20" s="9" t="s">
+        <v>84</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>12</v>
@@ -3506,9 +3487,8 @@
       <c r="F21" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="G21" s="9">
-        <f>IF(A21=1,"_",IF(C21="_","???",C21))</f>
-        <v/>
+      <c r="G21" s="9" t="s">
+        <v>88</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>12</v>
@@ -3537,9 +3517,8 @@
       <c r="F22" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="G22" s="9">
-        <f>IF(A22=1,"_",IF(C22="_","???",C22))</f>
-        <v/>
+      <c r="G22" s="9" t="s">
+        <v>92</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>12</v>
@@ -3568,9 +3547,8 @@
       <c r="F23" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="G23" s="9">
-        <f>IF(A23=1,"_",IF(C23="_","???",C23))</f>
-        <v/>
+      <c r="G23" s="9" t="s">
+        <v>96</v>
       </c>
       <c r="H23" s="10" t="s">
         <v>12</v>
@@ -3599,9 +3577,8 @@
       <c r="F24" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="G24" s="9">
-        <f>IF(A24=1,"_",IF(C24="_","???",C24))</f>
-        <v/>
+      <c r="G24" s="9" t="s">
+        <v>100</v>
       </c>
       <c r="H24" s="10" t="s">
         <v>12</v>
@@ -3630,9 +3607,8 @@
       <c r="F25" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="G25" s="9">
-        <f>IF(A25=1,"_",IF(C25="_","???",C25))</f>
-        <v/>
+      <c r="G25" s="9" t="s">
+        <v>104</v>
       </c>
       <c r="H25" s="10" t="s">
         <v>12</v>
@@ -3661,9 +3637,8 @@
       <c r="F26" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="G26" s="9">
-        <f>IF(A26=1,"_",IF(C26="_","???",C26))</f>
-        <v/>
+      <c r="G26" s="9" t="s">
+        <v>108</v>
       </c>
       <c r="H26" s="10" t="s">
         <v>12</v>
@@ -3692,9 +3667,8 @@
       <c r="F27" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="G27" s="9">
-        <f>IF(A27=1,"_",IF(C27="_","???",C27))</f>
-        <v/>
+      <c r="G27" s="9" t="s">
+        <v>112</v>
       </c>
       <c r="H27" s="10" t="s">
         <v>12</v>
@@ -3723,9 +3697,8 @@
       <c r="F28" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="G28" s="9">
-        <f>IF(A28=1,"_",IF(C28="_","???",C28))</f>
-        <v/>
+      <c r="G28" s="9" t="s">
+        <v>114</v>
       </c>
       <c r="H28" s="10" t="s">
         <v>12</v>
@@ -3754,9 +3727,8 @@
       <c r="F29" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="G29" s="9">
-        <f>IF(A29=1,"_",IF(C29="_","???",C29))</f>
-        <v/>
+      <c r="G29" s="9" t="s">
+        <v>117</v>
       </c>
       <c r="H29" s="10" t="s">
         <v>12</v>
@@ -3785,9 +3757,8 @@
       <c r="F30" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="G30" s="9">
-        <f>IF(A30=1,"_",IF(C30="_","???",C30))</f>
-        <v/>
+      <c r="G30" s="9" t="s">
+        <v>121</v>
       </c>
       <c r="H30" s="10" t="s">
         <v>12</v>
@@ -3816,9 +3787,8 @@
       <c r="F31" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="G31" s="9">
-        <f>IF(A31=1,"_",IF(C31="_","???",C31))</f>
-        <v/>
+      <c r="G31" s="9" t="s">
+        <v>124</v>
       </c>
       <c r="H31" s="10" t="s">
         <v>12</v>
@@ -3847,9 +3817,8 @@
       <c r="F32" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="G32" s="9">
-        <f>IF(A32=1,"_",IF(C32="_","???",C32))</f>
-        <v/>
+      <c r="G32" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="H32" s="10" t="s">
         <v>12</v>
@@ -3878,9 +3847,8 @@
       <c r="F33" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="G33" s="9">
-        <f>IF(A33=1,"_",IF(C33="_","???",C33))</f>
-        <v/>
+      <c r="G33" s="9" t="s">
+        <v>131</v>
       </c>
       <c r="H33" s="10" t="s">
         <v>12</v>
@@ -3909,9 +3877,8 @@
       <c r="F34" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="G34" s="9">
-        <f>IF(A34=1,"_",IF(C34="_","???",C34))</f>
-        <v/>
+      <c r="G34" s="9" t="s">
+        <v>135</v>
       </c>
       <c r="H34" s="10" t="s">
         <v>12</v>
@@ -3940,9 +3907,8 @@
       <c r="F35" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="G35" s="9">
-        <f>IF(A35=1,"_",IF(C35="_","???",C35))</f>
-        <v/>
+      <c r="G35" s="9" t="s">
+        <v>139</v>
       </c>
       <c r="H35" s="10" t="s">
         <v>12</v>
@@ -3971,9 +3937,8 @@
       <c r="F36" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="G36" s="9">
-        <f>IF(A36=1,"_",IF(C36="_","???",C36))</f>
-        <v/>
+      <c r="G36" s="9" t="s">
+        <v>143</v>
       </c>
       <c r="H36" s="10" t="s">
         <v>12</v>
@@ -4002,9 +3967,8 @@
       <c r="F37" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="G37" s="9">
-        <f>IF(A37=1,"_",IF(C37="_","???",C37))</f>
-        <v/>
+      <c r="G37" s="9" t="s">
+        <v>147</v>
       </c>
       <c r="H37" s="10" t="s">
         <v>12</v>
@@ -4033,9 +3997,8 @@
       <c r="F38" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="G38" s="9">
-        <f>IF(A38=1,"_",IF(C38="_","???",C38))</f>
-        <v/>
+      <c r="G38" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="H38" s="10" t="s">
         <v>12</v>
@@ -4064,9 +4027,8 @@
       <c r="F39" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="G39" s="9">
-        <f>IF(A39=1,"_",IF(C39="_","???",C39))</f>
-        <v/>
+      <c r="G39" s="9" t="s">
+        <v>154</v>
       </c>
       <c r="H39" s="10" t="s">
         <v>12</v>
@@ -4095,9 +4057,8 @@
       <c r="F40" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="G40" s="9">
-        <f>IF(A40=1,"_",IF(C40="_","???",C40))</f>
-        <v/>
+      <c r="G40" s="9" t="s">
+        <v>157</v>
       </c>
       <c r="H40" s="10" t="s">
         <v>12</v>
@@ -4126,9 +4087,8 @@
       <c r="F41" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="G41" s="9">
-        <f>IF(A41=1,"_",IF(C41="_","???",C41))</f>
-        <v/>
+      <c r="G41" s="9" t="s">
+        <v>161</v>
       </c>
       <c r="H41" s="10" t="s">
         <v>12</v>
@@ -4157,9 +4117,8 @@
       <c r="F42" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="G42" s="9">
-        <f>IF(A42=1,"_",IF(C42="_","???",C42))</f>
-        <v/>
+      <c r="G42" s="9" t="s">
+        <v>165</v>
       </c>
       <c r="H42" s="10" t="s">
         <v>12</v>
@@ -4188,9 +4147,8 @@
       <c r="F43" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="G43" s="9">
-        <f>IF(A43=1,"_",IF(C43="_","???",C43))</f>
-        <v/>
+      <c r="G43" s="9" t="s">
+        <v>168</v>
       </c>
       <c r="H43" s="10" t="s">
         <v>12</v>
@@ -4219,9 +4177,8 @@
       <c r="F44" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="G44" s="9">
-        <f>IF(A44=1,"_",IF(C44="_","???",C44))</f>
-        <v/>
+      <c r="G44" s="9" t="s">
+        <v>172</v>
       </c>
       <c r="H44" s="10" t="s">
         <v>12</v>
@@ -4250,9 +4207,8 @@
       <c r="F45" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="G45" s="9">
-        <f>IF(A45=1,"_",IF(C45="_","???",C45))</f>
-        <v/>
+      <c r="G45" s="9" t="s">
+        <v>176</v>
       </c>
       <c r="H45" s="10" t="s">
         <v>12</v>
@@ -4281,9 +4237,8 @@
       <c r="F46" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="G46" s="9">
-        <f>IF(A46=1,"_",IF(C46="_","???",C46))</f>
-        <v/>
+      <c r="G46" s="9" t="s">
+        <v>180</v>
       </c>
       <c r="H46" s="10" t="s">
         <v>12</v>
@@ -4312,9 +4267,8 @@
       <c r="F47" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="G47" s="9">
-        <f>IF(A47=1,"_",IF(C47="_","???",C47))</f>
-        <v/>
+      <c r="G47" s="9" t="s">
+        <v>182</v>
       </c>
       <c r="H47" s="10" t="s">
         <v>12</v>
@@ -4343,9 +4297,8 @@
       <c r="F48" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="G48" s="9">
-        <f>IF(A48=1,"_",IF(C48="_","???",C48))</f>
-        <v/>
+      <c r="G48" s="9" t="s">
+        <v>186</v>
       </c>
       <c r="H48" s="10" t="s">
         <v>12</v>
@@ -4374,9 +4327,8 @@
       <c r="F49" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="G49" s="9">
-        <f>IF(A49=1,"_",IF(C49="_","???",C49))</f>
-        <v/>
+      <c r="G49" s="9" t="s">
+        <v>190</v>
       </c>
       <c r="H49" s="10" t="s">
         <v>12</v>
@@ -4405,9 +4357,8 @@
       <c r="F50" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="G50" s="9">
-        <f>IF(A50=1,"_",IF(C50="_","???",C50))</f>
-        <v/>
+      <c r="G50" s="9" t="s">
+        <v>194</v>
       </c>
       <c r="H50" s="10" t="s">
         <v>12</v>
@@ -4436,9 +4387,8 @@
       <c r="F51" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="G51" s="9">
-        <f>IF(A51=1,"_",IF(C51="_","???",C51))</f>
-        <v/>
+      <c r="G51" s="9" t="s">
+        <v>198</v>
       </c>
       <c r="H51" s="10" t="s">
         <v>12</v>
@@ -4467,9 +4417,8 @@
       <c r="F52" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="G52" s="9">
-        <f>IF(A52=1,"_",IF(C52="_","???",C52))</f>
-        <v/>
+      <c r="G52" s="9" t="s">
+        <v>202</v>
       </c>
       <c r="H52" s="10" t="s">
         <v>12</v>
@@ -4498,9 +4447,8 @@
       <c r="F53" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="G53" s="9">
-        <f>IF(A53=1,"_",IF(C53="_","???",C53))</f>
-        <v/>
+      <c r="G53" s="9" t="s">
+        <v>206</v>
       </c>
       <c r="H53" s="10" t="s">
         <v>12</v>
@@ -4529,9 +4477,8 @@
       <c r="F54" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="G54" s="9">
-        <f>IF(A54=1,"_",IF(C54="_","???",C54))</f>
-        <v/>
+      <c r="G54" s="9" t="s">
+        <v>210</v>
       </c>
       <c r="H54" s="10" t="s">
         <v>12</v>
@@ -4560,9 +4507,8 @@
       <c r="F55" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="G55" s="9">
-        <f>IF(A55=1,"_",IF(C55="_","???",C55))</f>
-        <v/>
+      <c r="G55" s="9" t="s">
+        <v>213</v>
       </c>
       <c r="H55" s="10" t="s">
         <v>12</v>
@@ -4591,9 +4537,8 @@
       <c r="F56" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="G56" s="9">
-        <f>IF(A56=1,"_",IF(C56="_","???",C56))</f>
-        <v/>
+      <c r="G56" s="9" t="s">
+        <v>216</v>
       </c>
       <c r="H56" s="10" t="s">
         <v>12</v>
@@ -4622,9 +4567,8 @@
       <c r="F57" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="G57" s="9">
-        <f>IF(A57=1,"_",IF(C57="_","???",C57))</f>
-        <v/>
+      <c r="G57" s="9" t="s">
+        <v>220</v>
       </c>
       <c r="H57" s="10" t="s">
         <v>12</v>
@@ -4653,9 +4597,8 @@
       <c r="F58" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="G58" s="9">
-        <f>IF(A58=1,"_",IF(C58="_","???",C58))</f>
-        <v/>
+      <c r="G58" s="9" t="s">
+        <v>224</v>
       </c>
       <c r="H58" s="10" t="s">
         <v>12</v>
@@ -4684,9 +4627,8 @@
       <c r="F59" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="G59" s="9">
-        <f>IF(A59=1,"_",IF(C59="_","???",C59))</f>
-        <v/>
+      <c r="G59" s="9" t="s">
+        <v>227</v>
       </c>
       <c r="H59" s="10" t="s">
         <v>12</v>
@@ -4715,9 +4657,8 @@
       <c r="F60" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="G60" s="9">
-        <f>IF(A60=1,"_",IF(C60="_","???",C60))</f>
-        <v/>
+      <c r="G60" s="9" t="s">
+        <v>230</v>
       </c>
       <c r="H60" s="10" t="s">
         <v>12</v>
@@ -4746,9 +4687,8 @@
       <c r="F61" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="G61" s="9">
-        <f>IF(A61=1,"_",IF(C61="_","???",C61))</f>
-        <v/>
+      <c r="G61" s="9" t="s">
+        <v>232</v>
       </c>
       <c r="H61" s="10" t="s">
         <v>12</v>
@@ -4777,9 +4717,8 @@
       <c r="F62" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="G62" s="9">
-        <f>IF(A62=1,"_",IF(C62="_","???",C62))</f>
-        <v/>
+      <c r="G62" s="9" t="s">
+        <v>236</v>
       </c>
       <c r="H62" s="10" t="s">
         <v>12</v>
@@ -4808,9 +4747,8 @@
       <c r="F63" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="G63" s="9">
-        <f>IF(A63=1,"_",IF(C63="_","???",C63))</f>
-        <v/>
+      <c r="G63" s="9" t="s">
+        <v>239</v>
       </c>
       <c r="H63" s="10" t="s">
         <v>12</v>
@@ -4839,9 +4777,8 @@
       <c r="F64" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="G64" s="9">
-        <f>IF(A64=1,"_",IF(C64="_","???",C64))</f>
-        <v/>
+      <c r="G64" s="9" t="s">
+        <v>242</v>
       </c>
       <c r="H64" s="10" t="s">
         <v>12</v>
@@ -4870,9 +4807,8 @@
       <c r="F65" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="G65" s="9">
-        <f>IF(A65=1,"_",IF(C65="_","???",C65))</f>
-        <v/>
+      <c r="G65" s="9" t="s">
+        <v>244</v>
       </c>
       <c r="H65" s="10" t="s">
         <v>12</v>
@@ -4901,9 +4837,8 @@
       <c r="F66" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="G66" s="9">
-        <f>IF(A66=1,"_",IF(C66="_","???",C66))</f>
-        <v/>
+      <c r="G66" s="9" t="s">
+        <v>247</v>
       </c>
       <c r="H66" s="10" t="s">
         <v>12</v>
@@ -4932,9 +4867,8 @@
       <c r="F67" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="G67" s="9">
-        <f>IF(A67=1,"_",IF(C67="_","???",C67))</f>
-        <v/>
+      <c r="G67" s="9" t="s">
+        <v>251</v>
       </c>
       <c r="H67" s="10" t="s">
         <v>12</v>
@@ -4963,9 +4897,8 @@
       <c r="F68" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="G68" s="9">
-        <f>IF(A68=1,"_",IF(C68="_","???",C68))</f>
-        <v/>
+      <c r="G68" s="9" t="s">
+        <v>255</v>
       </c>
       <c r="H68" s="10" t="s">
         <v>12</v>
@@ -4994,9 +4927,8 @@
       <c r="F69" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="G69" s="9">
-        <f>IF(A69=1,"_",IF(C69="_","???",C69))</f>
-        <v/>
+      <c r="G69" s="9" t="s">
+        <v>259</v>
       </c>
       <c r="H69" s="10" t="s">
         <v>12</v>
@@ -5025,9 +4957,8 @@
       <c r="F70" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="G70" s="9">
-        <f>IF(A70=1,"_",IF(C70="_","???",C70))</f>
-        <v/>
+      <c r="G70" s="9" t="s">
+        <v>261</v>
       </c>
       <c r="H70" s="10" t="s">
         <v>12</v>
@@ -5056,9 +4987,8 @@
       <c r="F71" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="G71" s="9">
-        <f>IF(A71=1,"_",IF(C71="_","???",C71))</f>
-        <v/>
+      <c r="G71" s="9" t="s">
+        <v>264</v>
       </c>
       <c r="H71" s="10" t="s">
         <v>12</v>
@@ -5087,9 +5017,8 @@
       <c r="F72" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="G72" s="9">
-        <f>IF(A72=1,"_",IF(C72="_","???",C72))</f>
-        <v/>
+      <c r="G72" s="9" t="s">
+        <v>267</v>
       </c>
       <c r="H72" s="10" t="s">
         <v>12</v>
@@ -5118,9 +5047,8 @@
       <c r="F73" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="G73" s="9">
-        <f>IF(A73=1,"_",IF(C73="_","???",C73))</f>
-        <v/>
+      <c r="G73" s="9" t="s">
+        <v>271</v>
       </c>
       <c r="H73" s="10" t="s">
         <v>12</v>
@@ -5149,9 +5077,8 @@
       <c r="F74" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="G74" s="9">
-        <f>IF(A74=1,"_",IF(C74="_","???",C74))</f>
-        <v/>
+      <c r="G74" s="9" t="s">
+        <v>275</v>
       </c>
       <c r="H74" s="10" t="s">
         <v>12</v>
@@ -5180,9 +5107,8 @@
       <c r="F75" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="G75" s="9">
-        <f>IF(A75=1,"_",IF(C75="_","???",C75))</f>
-        <v/>
+      <c r="G75" s="9" t="s">
+        <v>278</v>
       </c>
       <c r="H75" s="10" t="s">
         <v>12</v>
@@ -5211,9 +5137,8 @@
       <c r="F76" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="G76" s="9">
-        <f>IF(A76=1,"_",IF(C76="_","???",C76))</f>
-        <v/>
+      <c r="G76" s="9" t="s">
+        <v>282</v>
       </c>
       <c r="H76" s="10" t="s">
         <v>12</v>
@@ -5242,9 +5167,8 @@
       <c r="F77" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="G77" s="9">
-        <f>IF(A77=1,"_",IF(C77="_","???",C77))</f>
-        <v/>
+      <c r="G77" s="9" t="s">
+        <v>284</v>
       </c>
       <c r="H77" s="10" t="s">
         <v>12</v>
@@ -5273,9 +5197,8 @@
       <c r="F78" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="G78" s="9">
-        <f>IF(A78=1,"_",IF(C78="_","???",C78))</f>
-        <v/>
+      <c r="G78" s="9" t="s">
+        <v>287</v>
       </c>
       <c r="H78" s="10" t="s">
         <v>12</v>
@@ -5304,9 +5227,8 @@
       <c r="F79" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="G79" s="9">
-        <f>IF(A79=1,"_",IF(C79="_","???",C79))</f>
-        <v/>
+      <c r="G79" s="9" t="s">
+        <v>290</v>
       </c>
       <c r="H79" s="10" t="s">
         <v>12</v>
@@ -5335,9 +5257,8 @@
       <c r="F80" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="G80" s="9">
-        <f>IF(A80=1,"_",IF(C80="_","???",C80))</f>
-        <v/>
+      <c r="G80" s="9" t="s">
+        <v>293</v>
       </c>
       <c r="H80" s="10" t="s">
         <v>12</v>
@@ -5366,9 +5287,8 @@
       <c r="F81" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="G81" s="9">
-        <f>IF(A81=1,"_",IF(C81="_","???",C81))</f>
-        <v/>
+      <c r="G81" s="9" t="s">
+        <v>296</v>
       </c>
       <c r="H81" s="10" t="s">
         <v>12</v>
@@ -5397,9 +5317,8 @@
       <c r="F82" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="G82" s="9">
-        <f>IF(A82=1,"_",IF(C82="_","???",C82))</f>
-        <v/>
+      <c r="G82" s="9" t="s">
+        <v>299</v>
       </c>
       <c r="H82" s="10" t="s">
         <v>12</v>
@@ -5428,9 +5347,8 @@
       <c r="F83" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="G83" s="9">
-        <f>IF(A83=1,"_",IF(C83="_","???",C83))</f>
-        <v/>
+      <c r="G83" s="9" t="s">
+        <v>302</v>
       </c>
       <c r="H83" s="10" t="s">
         <v>12</v>
@@ -5459,9 +5377,8 @@
       <c r="F84" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="G84" s="9">
-        <f>IF(A84=1,"_",IF(C84="_","???",C84))</f>
-        <v/>
+      <c r="G84" s="9" t="s">
+        <v>305</v>
       </c>
       <c r="H84" s="10" t="s">
         <v>12</v>
@@ -5490,9 +5407,8 @@
       <c r="F85" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="G85" s="9">
-        <f>IF(A85=1,"_",IF(C85="_","???",C85))</f>
-        <v/>
+      <c r="G85" s="9" t="s">
+        <v>309</v>
       </c>
       <c r="H85" s="10" t="s">
         <v>12</v>
@@ -5521,9 +5437,8 @@
       <c r="F86" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="G86" s="9">
-        <f>IF(A86=1,"_",IF(C86="_","???",C86))</f>
-        <v/>
+      <c r="G86" s="9" t="s">
+        <v>313</v>
       </c>
       <c r="H86" s="10" t="s">
         <v>12</v>
@@ -5552,9 +5467,8 @@
       <c r="F87" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="G87" s="9">
-        <f>IF(A87=1,"_",IF(C87="_","???",C87))</f>
-        <v/>
+      <c r="G87" s="9" t="s">
+        <v>316</v>
       </c>
       <c r="H87" s="10" t="s">
         <v>12</v>
@@ -5583,9 +5497,8 @@
       <c r="F88" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="G88" s="9">
-        <f>IF(A88=1,"_",IF(C88="_","???",C88))</f>
-        <v/>
+      <c r="G88" s="9" t="s">
+        <v>320</v>
       </c>
       <c r="H88" s="10" t="s">
         <v>12</v>
@@ -5614,9 +5527,8 @@
       <c r="F89" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="G89" s="9">
-        <f>IF(A89=1,"_",IF(C89="_","???",C89))</f>
-        <v/>
+      <c r="G89" s="9" t="s">
+        <v>324</v>
       </c>
       <c r="H89" s="10" t="s">
         <v>12</v>
@@ -5645,9 +5557,8 @@
       <c r="F90" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="G90" s="9">
-        <f>IF(A90=1,"_",IF(C90="_","???",C90))</f>
-        <v/>
+      <c r="G90" s="9" t="s">
+        <v>328</v>
       </c>
       <c r="H90" s="10" t="s">
         <v>12</v>
@@ -5676,9 +5587,8 @@
       <c r="F91" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="G91" s="9">
-        <f>IF(A91=1,"_",IF(C91="_","???",C91))</f>
-        <v/>
+      <c r="G91" s="9" t="s">
+        <v>332</v>
       </c>
       <c r="H91" s="10" t="s">
         <v>12</v>
@@ -5707,9 +5617,8 @@
       <c r="F92" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="G92" s="9">
-        <f>IF(A92=1,"_",IF(C92="_","???",C92))</f>
-        <v/>
+      <c r="G92" s="9" t="s">
+        <v>336</v>
       </c>
       <c r="H92" s="10" t="s">
         <v>12</v>
@@ -5738,9 +5647,8 @@
       <c r="F93" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="G93" s="9">
-        <f>IF(A93=1,"_",IF(C93="_","???",C93))</f>
-        <v/>
+      <c r="G93" s="9" t="s">
+        <v>340</v>
       </c>
       <c r="H93" s="10" t="s">
         <v>12</v>
@@ -5769,9 +5677,8 @@
       <c r="F94" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="G94" s="9">
-        <f>IF(A94=1,"_",IF(C94="_","???",C94))</f>
-        <v/>
+      <c r="G94" s="9" t="s">
+        <v>344</v>
       </c>
       <c r="H94" s="10" t="s">
         <v>12</v>
@@ -5800,9 +5707,8 @@
       <c r="F95" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="G95" s="9">
-        <f>IF(A95=1,"_",IF(C95="_","???",C95))</f>
-        <v/>
+      <c r="G95" s="9" t="s">
+        <v>348</v>
       </c>
       <c r="H95" s="10" t="s">
         <v>12</v>
@@ -5831,9 +5737,8 @@
       <c r="F96" s="6" t="s">
         <v>352</v>
       </c>
-      <c r="G96" s="9">
-        <f>IF(A96=1,"_",IF(C96="_","???",C96))</f>
-        <v/>
+      <c r="G96" s="9" t="s">
+        <v>352</v>
       </c>
       <c r="H96" s="10" t="s">
         <v>12</v>

</xml_diff>